<commit_message>
feat: phase 2, AI layer with verifier and measured threshold, page and memo
Receipt reading, account suggestions from an enum and exception notes, all at build
time and cached in data/ai/. Verifier rejects figures, invented IDs and approval
claims. eval.json scores every step against the ground truth and picks the threshold.
Static page in site/ reads data/site/site.json. Memo and README are rendered from
templates so every number comes from data/.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/out/cierre_2026-09_andes_labs.xlsx
+++ b/data/out/cierre_2026-09_andes_labs.xlsx
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12">
@@ -566,7 +566,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>61</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13">
@@ -577,7 +577,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>IA no ejecutada</t>
+          <t>0.75</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>68</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15">
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>26626713.75</v>
+        <v>22744110.4</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>0</v>
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>25818734.75</v>
+        <v>26016104.75</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>0</v>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>14263666.85</v>
+        <v>14647522.1</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>0</v>
@@ -775,7 +775,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>10178995.6</v>
+        <v>10882931.25</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>0</v>
@@ -793,7 +793,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>103706000</v>
+        <v>105067844</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>0</v>
@@ -811,7 +811,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>16075880.1</v>
+        <v>16183534.75</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>0</v>
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>3671428.65</v>
+        <v>4166090.9</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>0</v>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>1586033.65</v>
+        <v>1725948.8</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>0</v>
@@ -856,16 +856,16 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>5.1.09</t>
+          <t>5.1.08</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Capacitación y suscripciones</t>
+          <t>Gastos de oficina y equipamiento menor</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>1113639.45</v>
+        <v>374862.35</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>0</v>
@@ -874,16 +874,16 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>5.1.10</t>
+          <t>5.1.09</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Comisiones y gastos bancarios</t>
+          <t>Capacitación y suscripciones</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>494719.25</v>
+        <v>1232143.5</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>0</v>
@@ -892,32 +892,50 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>5.2.01</t>
+          <t>5.1.10</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Diferencias de cambio</t>
+          <t>Comisiones y gastos bancarios</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>4781167.65</v>
+        <v>494719.25</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr"/>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>5.2.01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Diferencias de cambio</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>4781167.65</v>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr"/>
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Totales</t>
         </is>
       </c>
-      <c r="C16" s="4" t="n">
+      <c r="C17" s="4" t="n">
         <v>208316979.7</v>
       </c>
-      <c r="D16" s="4" t="n">
+      <c r="D17" s="4" t="n">
         <v>208316979.7</v>
       </c>
     </row>
@@ -1220,25 +1238,37 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>1.1.09</t>
+          <t>5.1.03</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Partidas pendientes de imputación</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr"/>
+          <t>Licencias de software</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>5.1.03</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Revisión humana</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
+          <t>IA (aceptada)</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>AI-0001</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>pending review</t>
+          <t>posted</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -1246,11 +1276,7 @@
           <t>RC-0206</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
+      <c r="Q4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1796,25 +1822,37 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>1.1.09</t>
+          <t>5.1.03</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Partidas pendientes de imputación</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr"/>
+          <t>Licencias de software</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>5.1.03</t>
+        </is>
+      </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Revisión humana</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
+          <t>IA (aceptada)</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>AI-0002</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>pending review</t>
+          <t>posted</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1822,11 +1860,7 @@
           <t>RC-0143</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
+      <c r="Q12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3321,25 +3355,37 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>1.1.09</t>
+          <t>5.1.01</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Partidas pendientes de imputación</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr"/>
+          <t>Publicidad y marketing</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>5.1.01</t>
+        </is>
+      </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Revisión humana</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
+          <t>IA (aceptada)</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>AI-0003</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>pending review</t>
+          <t>posted</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
@@ -3347,11 +3393,7 @@
           <t>RC-0207</t>
         </is>
       </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
+      <c r="Q33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3398,14 +3440,26 @@
           <t>Partidas pendientes de imputación</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>5.1.02</t>
+        </is>
+      </c>
       <c r="L34" t="inlineStr">
         <is>
           <t>Revisión humana</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>AI-0004</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>0.68</t>
+        </is>
+      </c>
       <c r="O34" t="inlineStr">
         <is>
           <t>pending review</t>
@@ -3414,7 +3468,7 @@
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>missing_receipt, no_rule</t>
+          <t>missing_receipt, ai_below_threshold</t>
         </is>
       </c>
     </row>
@@ -4485,14 +4539,26 @@
           <t>Partidas pendientes de imputación</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr"/>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>5.1.08</t>
+        </is>
+      </c>
       <c r="L49" t="inlineStr">
         <is>
           <t>Revisión humana</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>AI-0005</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>0.72</t>
+        </is>
+      </c>
       <c r="O49" t="inlineStr">
         <is>
           <t>pending review</t>
@@ -4505,7 +4571,7 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>no_rule</t>
+          <t>ai_below_threshold</t>
         </is>
       </c>
     </row>
@@ -4619,25 +4685,37 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>1.1.09</t>
+          <t>5.1.04</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>Partidas pendientes de imputación</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr"/>
+          <t>Honorarios de contratistas del exterior</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>5.1.04</t>
+        </is>
+      </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>Revisión humana</t>
-        </is>
-      </c>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
+          <t>IA (aceptada)</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>AI-0006</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>pending review</t>
+          <t>posted</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
@@ -4645,11 +4723,7 @@
           <t>RC-0026</t>
         </is>
       </c>
-      <c r="Q51" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
+      <c r="Q51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5272,25 +5346,37 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>1.1.09</t>
+          <t>5.1.07</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>Partidas pendientes de imputación</t>
-        </is>
-      </c>
-      <c r="K60" t="inlineStr"/>
+          <t>Eventos y conferencias</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>5.1.07</t>
+        </is>
+      </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>Revisión humana</t>
-        </is>
-      </c>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
+          <t>IA (aceptada)</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>AI-0007</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>pending review</t>
+          <t>posted</t>
         </is>
       </c>
       <c r="P60" t="inlineStr">
@@ -5298,11 +5384,7 @@
           <t>RC-0112</t>
         </is>
       </c>
-      <c r="Q60" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
+      <c r="Q60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5341,25 +5423,37 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>1.1.09</t>
+          <t>5.1.09</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>Partidas pendientes de imputación</t>
-        </is>
-      </c>
-      <c r="K61" t="inlineStr"/>
+          <t>Capacitación y suscripciones</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>5.1.09</t>
+        </is>
+      </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>Revisión humana</t>
-        </is>
-      </c>
-      <c r="M61" t="inlineStr"/>
-      <c r="N61" t="inlineStr"/>
+          <t>IA (aceptada)</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>AI-0008</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>0.90</t>
+        </is>
+      </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>pending review</t>
+          <t>posted</t>
         </is>
       </c>
       <c r="P61" t="inlineStr">
@@ -5367,11 +5461,7 @@
           <t>RC-0132</t>
         </is>
       </c>
-      <c r="Q61" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
+      <c r="Q61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -5556,25 +5646,37 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>1.1.09</t>
+          <t>5.1.09</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>Partidas pendientes de imputación</t>
-        </is>
-      </c>
-      <c r="K64" t="inlineStr"/>
+          <t>Capacitación y suscripciones</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>5.1.09</t>
+        </is>
+      </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>Revisión humana</t>
-        </is>
-      </c>
-      <c r="M64" t="inlineStr"/>
-      <c r="N64" t="inlineStr"/>
+          <t>IA (aceptada)</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>AI-0009</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>0.85</t>
+        </is>
+      </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>pending review</t>
+          <t>posted</t>
         </is>
       </c>
       <c r="P64" t="inlineStr">
@@ -5582,11 +5684,7 @@
           <t>RC-0085</t>
         </is>
       </c>
-      <c r="Q64" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
+      <c r="Q64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5706,14 +5804,26 @@
           <t>Partidas pendientes de imputación</t>
         </is>
       </c>
-      <c r="K66" t="inlineStr"/>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>5.1.04</t>
+        </is>
+      </c>
       <c r="L66" t="inlineStr">
         <is>
           <t>Revisión humana</t>
         </is>
       </c>
-      <c r="M66" t="inlineStr"/>
-      <c r="N66" t="inlineStr"/>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>AI-0010</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>0.40</t>
+        </is>
+      </c>
       <c r="O66" t="inlineStr">
         <is>
           <t>pending review</t>
@@ -5722,7 +5832,7 @@
       <c r="P66" t="inlineStr"/>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>missing_receipt, no_rule</t>
+          <t>missing_receipt, ai_below_threshold</t>
         </is>
       </c>
     </row>
@@ -9052,25 +9162,37 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>1.1.09</t>
+          <t>5.1.05</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>Partidas pendientes de imputación</t>
-        </is>
-      </c>
-      <c r="K112" t="inlineStr"/>
+          <t>Viajes y viáticos</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>5.1.05</t>
+        </is>
+      </c>
       <c r="L112" t="inlineStr">
         <is>
-          <t>Revisión humana</t>
-        </is>
-      </c>
-      <c r="M112" t="inlineStr"/>
-      <c r="N112" t="inlineStr"/>
+          <t>IA (aceptada)</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>AI-0011</t>
+        </is>
+      </c>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>pending review</t>
+          <t>posted</t>
         </is>
       </c>
       <c r="P112" t="inlineStr">
@@ -9078,11 +9200,7 @@
           <t>RC-0197</t>
         </is>
       </c>
-      <c r="Q112" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
+      <c r="Q112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -9348,14 +9466,26 @@
           <t>Partidas pendientes de imputación</t>
         </is>
       </c>
-      <c r="K116" t="inlineStr"/>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>5.1.06</t>
+        </is>
+      </c>
       <c r="L116" t="inlineStr">
         <is>
           <t>Revisión humana</t>
         </is>
       </c>
-      <c r="M116" t="inlineStr"/>
-      <c r="N116" t="inlineStr"/>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>AI-0012</t>
+        </is>
+      </c>
+      <c r="N116" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
       <c r="O116" t="inlineStr">
         <is>
           <t>pending review</t>
@@ -9364,7 +9494,7 @@
       <c r="P116" t="inlineStr"/>
       <c r="Q116" t="inlineStr">
         <is>
-          <t>missing_receipt, no_rule</t>
+          <t>missing_receipt</t>
         </is>
       </c>
     </row>
@@ -9405,25 +9535,37 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>1.1.09</t>
+          <t>5.1.06</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>Partidas pendientes de imputación</t>
-        </is>
-      </c>
-      <c r="K117" t="inlineStr"/>
+          <t>Comidas y representación</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>5.1.06</t>
+        </is>
+      </c>
       <c r="L117" t="inlineStr">
         <is>
-          <t>Revisión humana</t>
-        </is>
-      </c>
-      <c r="M117" t="inlineStr"/>
-      <c r="N117" t="inlineStr"/>
+          <t>IA (aceptada)</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>AI-0013</t>
+        </is>
+      </c>
+      <c r="N117" t="inlineStr">
+        <is>
+          <t>0.93</t>
+        </is>
+      </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>pending review</t>
+          <t>posted</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -9431,11 +9573,7 @@
           <t>RC-0093</t>
         </is>
       </c>
-      <c r="Q117" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
+      <c r="Q117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -10212,14 +10350,26 @@
           <t>Partidas pendientes de imputación</t>
         </is>
       </c>
-      <c r="K128" t="inlineStr"/>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>5.1.01</t>
+        </is>
+      </c>
       <c r="L128" t="inlineStr">
         <is>
           <t>Revisión humana</t>
         </is>
       </c>
-      <c r="M128" t="inlineStr"/>
-      <c r="N128" t="inlineStr"/>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>AI-0014</t>
+        </is>
+      </c>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t>0.72</t>
+        </is>
+      </c>
       <c r="O128" t="inlineStr">
         <is>
           <t>pending review</t>
@@ -10232,7 +10382,7 @@
       </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t>no_rule</t>
+          <t>ai_below_threshold</t>
         </is>
       </c>
     </row>
@@ -10715,25 +10865,37 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>1.1.09</t>
+          <t>5.1.06</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>Partidas pendientes de imputación</t>
-        </is>
-      </c>
-      <c r="K135" t="inlineStr"/>
+          <t>Comidas y representación</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>5.1.06</t>
+        </is>
+      </c>
       <c r="L135" t="inlineStr">
         <is>
-          <t>Revisión humana</t>
-        </is>
-      </c>
-      <c r="M135" t="inlineStr"/>
-      <c r="N135" t="inlineStr"/>
+          <t>IA (aceptada)</t>
+        </is>
+      </c>
+      <c r="M135" t="inlineStr">
+        <is>
+          <t>AI-0015</t>
+        </is>
+      </c>
+      <c r="N135" t="inlineStr">
+        <is>
+          <t>0.90</t>
+        </is>
+      </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>pending review</t>
+          <t>posted</t>
         </is>
       </c>
       <c r="P135" t="inlineStr">
@@ -10741,11 +10903,7 @@
           <t>RC-0161</t>
         </is>
       </c>
-      <c r="Q135" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
+      <c r="Q135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -11295,25 +11453,37 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>1.1.09</t>
+          <t>5.1.04</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>Partidas pendientes de imputación</t>
-        </is>
-      </c>
-      <c r="K143" t="inlineStr"/>
+          <t>Honorarios de contratistas del exterior</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>5.1.04</t>
+        </is>
+      </c>
       <c r="L143" t="inlineStr">
         <is>
-          <t>Revisión humana</t>
-        </is>
-      </c>
-      <c r="M143" t="inlineStr"/>
-      <c r="N143" t="inlineStr"/>
+          <t>IA (aceptada)</t>
+        </is>
+      </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>AI-0016</t>
+        </is>
+      </c>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
       <c r="O143" t="inlineStr">
         <is>
-          <t>pending review</t>
+          <t>posted</t>
         </is>
       </c>
       <c r="P143" t="inlineStr">
@@ -11321,11 +11491,7 @@
           <t>RC-0033</t>
         </is>
       </c>
-      <c r="Q143" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
+      <c r="Q143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -12317,25 +12483,37 @@
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>1.1.09</t>
+          <t>5.1.08</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>Partidas pendientes de imputación</t>
-        </is>
-      </c>
-      <c r="K157" t="inlineStr"/>
+          <t>Gastos de oficina y equipamiento menor</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>5.1.08</t>
+        </is>
+      </c>
       <c r="L157" t="inlineStr">
         <is>
-          <t>Revisión humana</t>
-        </is>
-      </c>
-      <c r="M157" t="inlineStr"/>
-      <c r="N157" t="inlineStr"/>
+          <t>IA (aceptada)</t>
+        </is>
+      </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>AI-0017</t>
+        </is>
+      </c>
+      <c r="N157" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>pending review</t>
+          <t>posted</t>
         </is>
       </c>
       <c r="P157" t="inlineStr">
@@ -12343,11 +12521,7 @@
           <t>RC-0167</t>
         </is>
       </c>
-      <c r="Q157" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
+      <c r="Q157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -12763,14 +12937,26 @@
           <t>Partidas pendientes de imputación</t>
         </is>
       </c>
-      <c r="K163" t="inlineStr"/>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>5.1.02</t>
+        </is>
+      </c>
       <c r="L163" t="inlineStr">
         <is>
           <t>Revisión humana</t>
         </is>
       </c>
-      <c r="M163" t="inlineStr"/>
-      <c r="N163" t="inlineStr"/>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>AI-0018</t>
+        </is>
+      </c>
+      <c r="N163" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
       <c r="O163" t="inlineStr">
         <is>
           <t>pending review</t>
@@ -12779,7 +12965,7 @@
       <c r="P163" t="inlineStr"/>
       <c r="Q163" t="inlineStr">
         <is>
-          <t>missing_receipt, no_rule</t>
+          <t>missing_receipt</t>
         </is>
       </c>
     </row>
@@ -13112,25 +13298,37 @@
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>1.1.09</t>
+          <t>5.1.08</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>Partidas pendientes de imputación</t>
-        </is>
-      </c>
-      <c r="K168" t="inlineStr"/>
+          <t>Gastos de oficina y equipamiento menor</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>5.1.08</t>
+        </is>
+      </c>
       <c r="L168" t="inlineStr">
         <is>
-          <t>Revisión humana</t>
-        </is>
-      </c>
-      <c r="M168" t="inlineStr"/>
-      <c r="N168" t="inlineStr"/>
+          <t>IA (aceptada)</t>
+        </is>
+      </c>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>AI-0019</t>
+        </is>
+      </c>
+      <c r="N168" t="inlineStr">
+        <is>
+          <t>0.90</t>
+        </is>
+      </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>pending review</t>
+          <t>posted</t>
         </is>
       </c>
       <c r="P168" t="inlineStr">
@@ -13138,11 +13336,7 @@
           <t>RC-0157</t>
         </is>
       </c>
-      <c r="Q168" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
+      <c r="Q168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -13331,25 +13525,37 @@
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>1.1.09</t>
+          <t>5.1.03</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>Partidas pendientes de imputación</t>
-        </is>
-      </c>
-      <c r="K171" t="inlineStr"/>
+          <t>Licencias de software</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>5.1.03</t>
+        </is>
+      </c>
       <c r="L171" t="inlineStr">
         <is>
-          <t>Revisión humana</t>
-        </is>
-      </c>
-      <c r="M171" t="inlineStr"/>
-      <c r="N171" t="inlineStr"/>
+          <t>IA (aceptada)</t>
+        </is>
+      </c>
+      <c r="M171" t="inlineStr">
+        <is>
+          <t>AI-0020</t>
+        </is>
+      </c>
+      <c r="N171" t="inlineStr">
+        <is>
+          <t>0.90</t>
+        </is>
+      </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>pending review</t>
+          <t>posted</t>
         </is>
       </c>
       <c r="P171" t="inlineStr">
@@ -13357,11 +13563,7 @@
           <t>RC-0129</t>
         </is>
       </c>
-      <c r="Q171" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
+      <c r="Q171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -13400,25 +13602,37 @@
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>1.1.09</t>
+          <t>5.1.05</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>Partidas pendientes de imputación</t>
-        </is>
-      </c>
-      <c r="K172" t="inlineStr"/>
+          <t>Viajes y viáticos</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>5.1.05</t>
+        </is>
+      </c>
       <c r="L172" t="inlineStr">
         <is>
-          <t>Revisión humana</t>
-        </is>
-      </c>
-      <c r="M172" t="inlineStr"/>
-      <c r="N172" t="inlineStr"/>
+          <t>IA (aceptada)</t>
+        </is>
+      </c>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>AI-0021</t>
+        </is>
+      </c>
+      <c r="N172" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t>pending review</t>
+          <t>posted</t>
         </is>
       </c>
       <c r="P172" t="inlineStr">
@@ -13426,11 +13640,7 @@
           <t>RC-0138</t>
         </is>
       </c>
-      <c r="Q172" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
+      <c r="Q172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -13907,25 +14117,37 @@
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>1.1.09</t>
+          <t>5.1.05</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>Partidas pendientes de imputación</t>
-        </is>
-      </c>
-      <c r="K179" t="inlineStr"/>
+          <t>Viajes y viáticos</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>5.1.05</t>
+        </is>
+      </c>
       <c r="L179" t="inlineStr">
         <is>
-          <t>Revisión humana</t>
-        </is>
-      </c>
-      <c r="M179" t="inlineStr"/>
-      <c r="N179" t="inlineStr"/>
+          <t>IA (aceptada)</t>
+        </is>
+      </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>AI-0022</t>
+        </is>
+      </c>
+      <c r="N179" t="inlineStr">
+        <is>
+          <t>0.85</t>
+        </is>
+      </c>
       <c r="O179" t="inlineStr">
         <is>
-          <t>pending review</t>
+          <t>posted</t>
         </is>
       </c>
       <c r="P179" t="inlineStr">
@@ -13933,11 +14155,7 @@
           <t>RC-0023</t>
         </is>
       </c>
-      <c r="Q179" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
+      <c r="Q179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -14637,14 +14855,26 @@
           <t>Partidas pendientes de imputación</t>
         </is>
       </c>
-      <c r="K189" t="inlineStr"/>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>5.1.01</t>
+        </is>
+      </c>
       <c r="L189" t="inlineStr">
         <is>
           <t>Revisión humana</t>
         </is>
       </c>
-      <c r="M189" t="inlineStr"/>
-      <c r="N189" t="inlineStr"/>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>AI-0023</t>
+        </is>
+      </c>
+      <c r="N189" t="inlineStr">
+        <is>
+          <t>0.60</t>
+        </is>
+      </c>
       <c r="O189" t="inlineStr">
         <is>
           <t>pending review</t>
@@ -14653,7 +14883,7 @@
       <c r="P189" t="inlineStr"/>
       <c r="Q189" t="inlineStr">
         <is>
-          <t>missing_receipt, no_rule</t>
+          <t>missing_receipt, ai_below_threshold</t>
         </is>
       </c>
     </row>
@@ -14694,25 +14924,37 @@
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>1.1.09</t>
+          <t>5.1.07</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>Partidas pendientes de imputación</t>
-        </is>
-      </c>
-      <c r="K190" t="inlineStr"/>
+          <t>Eventos y conferencias</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>5.1.07</t>
+        </is>
+      </c>
       <c r="L190" t="inlineStr">
         <is>
-          <t>Revisión humana</t>
-        </is>
-      </c>
-      <c r="M190" t="inlineStr"/>
-      <c r="N190" t="inlineStr"/>
+          <t>IA (aceptada)</t>
+        </is>
+      </c>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>AI-0024</t>
+        </is>
+      </c>
+      <c r="N190" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
       <c r="O190" t="inlineStr">
         <is>
-          <t>pending review</t>
+          <t>posted</t>
         </is>
       </c>
       <c r="P190" t="inlineStr">
@@ -14720,11 +14962,7 @@
           <t>RC-0163</t>
         </is>
       </c>
-      <c r="Q190" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
+      <c r="Q190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -15128,25 +15366,37 @@
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>1.1.09</t>
+          <t>5.1.06</t>
         </is>
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>Partidas pendientes de imputación</t>
-        </is>
-      </c>
-      <c r="K196" t="inlineStr"/>
+          <t>Comidas y representación</t>
+        </is>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>5.1.06</t>
+        </is>
+      </c>
       <c r="L196" t="inlineStr">
         <is>
-          <t>Revisión humana</t>
-        </is>
-      </c>
-      <c r="M196" t="inlineStr"/>
-      <c r="N196" t="inlineStr"/>
+          <t>IA (aceptada)</t>
+        </is>
+      </c>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>AI-0025</t>
+        </is>
+      </c>
+      <c r="N196" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
       <c r="O196" t="inlineStr">
         <is>
-          <t>pending review</t>
+          <t>posted</t>
         </is>
       </c>
       <c r="P196" t="inlineStr">
@@ -15154,11 +15404,7 @@
           <t>RC-0021</t>
         </is>
       </c>
-      <c r="Q196" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
+      <c r="Q196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -16081,14 +16327,26 @@
           <t>Partidas pendientes de imputación</t>
         </is>
       </c>
-      <c r="K209" t="inlineStr"/>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>5.1.06</t>
+        </is>
+      </c>
       <c r="L209" t="inlineStr">
         <is>
           <t>Revisión humana</t>
         </is>
       </c>
-      <c r="M209" t="inlineStr"/>
-      <c r="N209" t="inlineStr"/>
+      <c r="M209" t="inlineStr">
+        <is>
+          <t>AI-0026</t>
+        </is>
+      </c>
+      <c r="N209" t="inlineStr">
+        <is>
+          <t>0.85</t>
+        </is>
+      </c>
       <c r="O209" t="inlineStr">
         <is>
           <t>pending review</t>
@@ -16097,7 +16355,7 @@
       <c r="P209" t="inlineStr"/>
       <c r="Q209" t="inlineStr">
         <is>
-          <t>missing_receipt, no_rule</t>
+          <t>missing_receipt</t>
         </is>
       </c>
     </row>
@@ -16511,14 +16769,26 @@
           <t>Partidas pendientes de imputación</t>
         </is>
       </c>
-      <c r="K215" t="inlineStr"/>
+      <c r="K215" t="inlineStr">
+        <is>
+          <t>5.1.03</t>
+        </is>
+      </c>
       <c r="L215" t="inlineStr">
         <is>
           <t>Revisión humana</t>
         </is>
       </c>
-      <c r="M215" t="inlineStr"/>
-      <c r="N215" t="inlineStr"/>
+      <c r="M215" t="inlineStr">
+        <is>
+          <t>AI-0027</t>
+        </is>
+      </c>
+      <c r="N215" t="inlineStr">
+        <is>
+          <t>0.72</t>
+        </is>
+      </c>
       <c r="O215" t="inlineStr">
         <is>
           <t>pending review</t>
@@ -16531,7 +16801,7 @@
       </c>
       <c r="Q215" t="inlineStr">
         <is>
-          <t>no_rule</t>
+          <t>ai_below_threshold</t>
         </is>
       </c>
     </row>
@@ -17590,25 +17860,37 @@
       </c>
       <c r="I230" t="inlineStr">
         <is>
-          <t>1.1.09</t>
+          <t>5.1.02</t>
         </is>
       </c>
       <c r="J230" t="inlineStr">
         <is>
-          <t>Partidas pendientes de imputación</t>
-        </is>
-      </c>
-      <c r="K230" t="inlineStr"/>
+          <t>Servicios de nube</t>
+        </is>
+      </c>
+      <c r="K230" t="inlineStr">
+        <is>
+          <t>5.1.02</t>
+        </is>
+      </c>
       <c r="L230" t="inlineStr">
         <is>
-          <t>Revisión humana</t>
-        </is>
-      </c>
-      <c r="M230" t="inlineStr"/>
-      <c r="N230" t="inlineStr"/>
+          <t>IA (aceptada)</t>
+        </is>
+      </c>
+      <c r="M230" t="inlineStr">
+        <is>
+          <t>AI-0028</t>
+        </is>
+      </c>
+      <c r="N230" t="inlineStr">
+        <is>
+          <t>0.85</t>
+        </is>
+      </c>
       <c r="O230" t="inlineStr">
         <is>
-          <t>pending review</t>
+          <t>posted</t>
         </is>
       </c>
       <c r="P230" t="inlineStr">
@@ -17616,11 +17898,7 @@
           <t>RC-0154</t>
         </is>
       </c>
-      <c r="Q230" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
+      <c r="Q230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -18316,25 +18594,37 @@
       </c>
       <c r="I240" t="inlineStr">
         <is>
-          <t>1.1.09</t>
+          <t>5.1.09</t>
         </is>
       </c>
       <c r="J240" t="inlineStr">
         <is>
-          <t>Partidas pendientes de imputación</t>
-        </is>
-      </c>
-      <c r="K240" t="inlineStr"/>
+          <t>Capacitación y suscripciones</t>
+        </is>
+      </c>
+      <c r="K240" t="inlineStr">
+        <is>
+          <t>5.1.09</t>
+        </is>
+      </c>
       <c r="L240" t="inlineStr">
         <is>
-          <t>Revisión humana</t>
-        </is>
-      </c>
-      <c r="M240" t="inlineStr"/>
-      <c r="N240" t="inlineStr"/>
+          <t>IA (aceptada)</t>
+        </is>
+      </c>
+      <c r="M240" t="inlineStr">
+        <is>
+          <t>AI-0029</t>
+        </is>
+      </c>
+      <c r="N240" t="inlineStr">
+        <is>
+          <t>0.85</t>
+        </is>
+      </c>
       <c r="O240" t="inlineStr">
         <is>
-          <t>pending review</t>
+          <t>posted</t>
         </is>
       </c>
       <c r="P240" t="inlineStr">
@@ -18342,11 +18632,7 @@
           <t>RC-0122</t>
         </is>
       </c>
-      <c r="Q240" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
+      <c r="Q240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -18673,25 +18959,37 @@
       </c>
       <c r="I245" t="inlineStr">
         <is>
-          <t>1.1.09</t>
+          <t>5.1.02</t>
         </is>
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>Partidas pendientes de imputación</t>
-        </is>
-      </c>
-      <c r="K245" t="inlineStr"/>
+          <t>Servicios de nube</t>
+        </is>
+      </c>
+      <c r="K245" t="inlineStr">
+        <is>
+          <t>5.1.02</t>
+        </is>
+      </c>
       <c r="L245" t="inlineStr">
         <is>
-          <t>Revisión humana</t>
-        </is>
-      </c>
-      <c r="M245" t="inlineStr"/>
-      <c r="N245" t="inlineStr"/>
+          <t>IA (aceptada)</t>
+        </is>
+      </c>
+      <c r="M245" t="inlineStr">
+        <is>
+          <t>AI-0030</t>
+        </is>
+      </c>
+      <c r="N245" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
       <c r="O245" t="inlineStr">
         <is>
-          <t>pending review</t>
+          <t>posted</t>
         </is>
       </c>
       <c r="P245" t="inlineStr">
@@ -18699,11 +18997,7 @@
           <t>RC-0213</t>
         </is>
       </c>
-      <c r="Q245" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
+      <c r="Q245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -19300,7 +19594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -19357,28 +19651,28 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>no_rule</t>
+          <t>missing_receipt</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>TX-0003</t>
+          <t>TX-0005</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>TX-0003 · 2026-09-01 · PADDLE.NET* SCREENSTUDIO · USD 91.26 · Sofía Paz · no account rule matches the descriptor</t>
+          <t>TX-0005 · 2026-09-01 · TST* LA MAR CEBICHERIA · USD 73.22 · Camila Ortiz · no receipt found in the matching window</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>No rule covers the merchant of [TX-0003].</t>
+          <t>This restaurant card charge [TX-0005] has no receipt in the matching window, so there is no support for it yet. Ask the cardholder for the receipt and the business purpose, and check whether it was filed under a different date or card.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -19395,23 +19689,23 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>TX-0005</t>
+          <t>TX-0021</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>TX-0005 · 2026-09-01 · TST* LA MAR CEBICHERIA · USD 73.22 · Camila Ortiz · no receipt found in the matching window</t>
+          <t>TX-0021 · 2026-09-03 · TST* TARTINE BAKERY · USD 27.40 · Camila Ortiz · no receipt found in the matching window</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>No receipt was found for [TX-0005]. It stays in review until the cardholder uploads one.</t>
+          <t>The bakery card charge [TX-0021] has no receipt in the matching window, so there is no support for it yet. Ask the cardholder for the receipt and check whether it was filed under a different charge or sent late.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -19423,28 +19717,28 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>no_rule</t>
+          <t>missing_receipt</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>TX-0011</t>
+          <t>TX-0028</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>TX-0011 · 2026-09-02 · CALENDLY · USD 68.33 · Camila Ortiz · no account rule matches the descriptor</t>
+          <t>TX-0028 · 2026-09-04 · UBER *TRIP 66CTP · USD 20.71 · Julián Castro · no receipt found in the matching window</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>No rule covers the merchant of [TX-0011].</t>
+          <t>The ride charge [TX-0028] has no matching receipt in the expected window, so there is no support for it. Ask the cardholder for the receipt and confirm the trip was for business.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -19461,23 +19755,23 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>TX-0021</t>
+          <t>TX-0033</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>TX-0021 · 2026-09-03 · TST* TARTINE BAKERY · USD 27.40 · Camila Ortiz · no receipt found in the matching window</t>
+          <t>TX-0033 · 2026-09-05 · NAMECHEAP.COM · USD 68.99 · Martín Ibarra · no receipt found in the matching window</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>No receipt was found for [TX-0021]. It stays in review until the cardholder uploads one.</t>
+          <t>The card charge [TX-0033] from Namecheap has no receipt, so we can't tell if it was a domain, hosting, an SSL certificate or something else. Ask the cardholder for the receipt before relying on the cloud services suggestion [AI-0004], since that account is only a guess.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -19489,28 +19783,28 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>missing_receipt</t>
+          <t>ai_below_threshold</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>TX-0028</t>
+          <t>TX-0033</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>TX-0028 · 2026-09-04 · UBER *TRIP 66CTP · USD 20.71 · Julián Castro · no receipt found in the matching window</t>
+          <t>TX-0033 · 2026-09-05 · NAMECHEAP.COM · USD 68.99 · Martín Ibarra · AI suggests 5.1.02 Servicios de nube with confidence 0.68 · threshold 0.75</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>No receipt was found for [TX-0028]. It stays in review until the cardholder uploads one.</t>
+          <t>The AI's cloud services suggestion [AI-0004] for this Namecheap charge [TX-0033] is not confident enough to accept, and no receipt is matched. Find the invoice or ask the cardholder what was bought, since it could be a domain, hosting, a certificate or email, then pick the account.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -19522,28 +19816,28 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>no_rule</t>
+          <t>missing_receipt</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>TX-0032</t>
+          <t>TX-0038</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>TX-0032 · 2026-09-05 · BETALIST · USD 129.00 · Julián Castro · no account rule matches the descriptor</t>
+          <t>TX-0038 · 2026-09-06 · TST* SWEETGREEN MARKET  · USD 127.14 · Diego Romero · no receipt found in the matching window</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>No rule covers the merchant of [TX-0032].</t>
+          <t>This card charge [TX-0038] at a restaurant has no receipt in the matching window. Ask the cardholder for the receipt and check whether it was filed late or under a different charge.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -19555,28 +19849,28 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>missing_receipt</t>
+          <t>ai_below_threshold</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>TX-0033</t>
+          <t>TX-0048</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>TX-0033 · 2026-09-05 · NAMECHEAP.COM · USD 68.99 · Martín Ibarra · no receipt found in the matching window</t>
+          <t>TX-0048 · 2026-09-07 · WEWORK MEXICO · USD 42.95 · Valentina Sosa · AI suggests 5.1.08 Gastos de oficina y equipamiento menor with confidence 0.72 · threshold 0.75</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>No receipt was found for [TX-0033]. It stays in review until the cardholder uploads one.</t>
+          <t>The AI suggests office expenses for this coworking charge [TX-0048], but its confidence is under the threshold because the memo mentions a trip to Sao Paulo while the receipt [RC-0146] is from Mexico City. Check the receipt and ask the cardholder whether this was travel or office space, then pick the account (see AI-0005).</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -19588,28 +19882,28 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>no_rule</t>
+          <t>refund_partial_link</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>TX-0033</t>
+          <t>TX-0049</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>TX-0033 · 2026-09-05 · NAMECHEAP.COM · USD 68.99 · Martín Ibarra · no account rule matches the descriptor</t>
+          <t>TX-0049 · 2026-09-08 · BOOKING.COM HOTEL · USD 210.00 · Valentina Sosa · tentatively linked to TX-0024 posted 2026-09-04 for USD 239.51 · amounts differ</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>No rule covers the merchant of [TX-0033].</t>
+          <t>This refund [TX-0049] was matched to the earlier charge [TX-0024] only because the merchant name is the same, and the amounts don't agree, so it may be a partial refund or belong to a different booking. Check the booking details to confirm which charge [TX-0049] actually refunds, and whether [TX-0024] has any balance left over.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -19621,28 +19915,28 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>missing_receipt</t>
+          <t>duplicate_suspected</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>TX-0038</t>
+          <t>TX-0057</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>TX-0038 · 2026-09-06 · TST* SWEETGREEN MARKET  · USD 127.14 · Diego Romero · no receipt found in the matching window</t>
+          <t>TX-0057 · 2026-09-08 · UBER *TRIP TQ72G · USD 42.94 · Martín Ibarra · same descriptor and amount as TX-0056 posted 2026-09-08 · only one receipt</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>No receipt was found for [TX-0038]. It stays in review until the cardholder uploads one.</t>
+          <t>[TX-0057] has the same merchant descriptor and amount as [TX-0056], posted the same day, and only a single receipt backs the pair, so it may be a repeat charge. Check with the cardholder whether separate trips took place, and dispute [TX-0057] if they did not.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -19654,28 +19948,28 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>no_rule</t>
+          <t>missing_receipt</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>TX-0048</t>
+          <t>TX-0064</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>TX-0048 · 2026-09-07 · WEWORK MEXICO · USD 42.95 · Valentina Sosa · no account rule matches the descriptor</t>
+          <t>TX-0064 · 2026-09-10 · LINEAR ORBIT · USD 197.14 · Tomás Herrera · no receipt found in the matching window</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>No rule covers the merchant of [TX-0048].</t>
+          <t>The card charge [TX-0064] to Linear Orbit has no receipt in the matching window, so there is no support for it. Ask the cardholder for the receipt and check whether it was filed late or under a different charge.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -19687,28 +19981,28 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>refund_partial_link</t>
+          <t>missing_receipt</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>TX-0049</t>
+          <t>TX-0065</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>TX-0049 · 2026-09-08 · BOOKING.COM HOTEL · USD 210.00 · Valentina Sosa · tentatively linked to TX-0024 posted 2026-09-04 for USD 239.51 · amounts differ</t>
+          <t>TX-0065 · 2026-09-10 · PAYPAL *MGOMEZSTUDIO · USD 588.58 · Sofía Paz · no receipt found in the matching window</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[TX-0049] is a partial refund. It was linked to [TX-0024] because the merchant matches, but the amounts differ, so the link needs a person to confirm it.</t>
+          <t>The PayPal charge [TX-0065] has no receipt, and the payee looks like an individual or studio, so the suggested contractor account [AI-0010] is only a guess. Ask the cardholder for the receipt or invoice and confirm whether this was a contractor payment or a software or design purchase before accepting [AI-0010].</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -19720,28 +20014,28 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>no_rule</t>
+          <t>ai_below_threshold</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>TX-0050</t>
+          <t>TX-0065</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>TX-0050 · 2026-09-08 · FIVERR · USD 204.22 · Sofía Paz · no account rule matches the descriptor</t>
+          <t>TX-0065 · 2026-09-10 · PAYPAL *MGOMEZSTUDIO · USD 588.58 · Sofía Paz · AI suggests 5.1.04 Honorarios de contratistas del exterior with confidence 0.40 · threshold 0.75</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>No rule covers the merchant of [TX-0050].</t>
+          <t>The AI's contractor-fee suggestion [AI-0010] for this PayPal charge [TX-0065] is a weak guess, and no receipt or memo supports it. Confirm with the cardholder what was bought, and whether it was a freelancer or a software or design purchase, before choosing the account.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -19753,28 +20047,28 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>duplicate_suspected</t>
+          <t>missing_receipt</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>TX-0057</t>
+          <t>TX-0067</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>TX-0057 · 2026-09-08 · UBER *TRIP TQ72G · USD 42.94 · Martín Ibarra · same descriptor and amount as TX-0056 posted 2026-09-08 · only one receipt</t>
+          <t>TX-0067 · 2026-09-10 · TST* JOES PIZZA · USD 77.73 · Camila Ortiz · no receipt found in the matching window</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[TX-0057] repeats the merchant and amount of [TX-0056] within a short window, and only one receipt exists. It looks like a double charge.</t>
+          <t>The card charge [TX-0067] at a pizza restaurant has no receipt in the matching window. Ask the cardholder for the receipt and check whether it was filed late or under a different charge.</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -19786,28 +20080,28 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>no_rule</t>
+          <t>missing_receipt</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>TX-0059</t>
+          <t>TX-0069</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>TX-0059 · 2026-09-09 · SQ *SF DEVS MEETUP · USD 43.00 · Valentina Sosa · no account rule matches the descriptor</t>
+          <t>TX-0069 · 2026-09-10 · UBER *EATS HC9E7 · USD 50.39 · Tomás Herrera · no receipt found in the matching window</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>No rule covers the merchant of [TX-0059].</t>
+          <t>The food delivery charge [TX-0069] on Tomás Herrera's card has no receipt in the matching window. Ask the cardholder for the receipt and check that it was a business expense.</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -19819,28 +20113,28 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>no_rule</t>
+          <t>missing_receipt</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>TX-0060</t>
+          <t>TX-0071</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>TX-0060 · 2026-09-09 · THE ECONOMIST · USD 21.99 · Lucía Fernández · no account rule matches the descriptor</t>
+          <t>TX-0071 · 2026-09-10 · UBER *TRIP T386M · USD 18.81 · Julián Castro · no receipt found in the matching window</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>No rule covers the merchant of [TX-0060].</t>
+          <t>The ride-share charge [TX-0071] has no receipt in the matching window, so there is no support for it yet. Ask the cardholder for the receipt and confirm the trip was for business.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -19852,28 +20146,28 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>no_rule</t>
+          <t>amount_mismatch</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>TX-0063</t>
+          <t>TX-0072</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>TX-0063 · 2026-09-10 · GUMROAD.COM* SHAPEUP · USD 25.47 · Tomás Herrera · no account rule matches the descriptor</t>
+          <t>TX-0072 · 2026-09-10 · WEB SUMMIT RIO · USD 700.96 · Sofía Paz · receipt RC-0103 shows EUR 644.00 · different currency</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>No rule covers the merchant of [TX-0063].</t>
+          <t>The card charge [TX-0072] was billed in a different currency from the receipt [RC-0103], so the amounts can't be compared directly. Check whether [RC-0103] is the final receipt for this purchase and whether the gap comes only from exchange rate or fees, or ask Sofía Paz for the final receipt.</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -19890,23 +20184,23 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>TX-0064</t>
+          <t>TX-0073</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>TX-0064 · 2026-09-10 · LINEAR ORBIT · USD 197.14 · Tomás Herrera · no receipt found in the matching window</t>
+          <t>TX-0073 · 2026-09-11 · ATLASSIAN · USD 100.98 · Diego Romero · no receipt found in the matching window</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>No receipt was found for [TX-0064]. It stays in review until the cardholder uploads one.</t>
+          <t>The Atlassian card charge [TX-0073] has no receipt in the matching window, so there is no support for it yet. Ask the cardholder, Diego Romero, for the receipt and check whether it was filed late or under a different charge.</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -19918,28 +20212,28 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>missing_receipt</t>
+          <t>amount_mismatch</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>TX-0065</t>
+          <t>TX-0079</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>TX-0065 · 2026-09-10 · PAYPAL *MGOMEZSTUDIO · USD 588.58 · Sofía Paz · no receipt found in the matching window</t>
+          <t>TX-0079 · 2026-09-11 · MARRIOTT SAO PAULO · USD 333.76 · Valentina Sosa · receipt RC-0192 shows USD 293.76 · difference USD 40.00</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>No receipt was found for [TX-0065]. It stays in review until the cardholder uploads one.</t>
+          <t>The hotel charge [TX-0079] is higher than the amount on the receipt [RC-0192], so the receipt may not be the final bill. Check whether a final folio exists, for example with added extras or a later adjustment, or record the difference as unsupported.</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -19951,28 +20245,28 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>no_rule</t>
+          <t>refund_partial_link</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>TX-0065</t>
+          <t>TX-0083</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>TX-0065 · 2026-09-10 · PAYPAL *MGOMEZSTUDIO · USD 588.58 · Sofía Paz · no account rule matches the descriptor</t>
+          <t>TX-0083 · 2026-09-12 · AIRBNB * HMM7983 · USD 111.51 · Diego Romero · tentatively linked to TX-0061 posted 2026-09-10 for USD 743.41 · amounts differ</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>No rule covers the merchant of [TX-0065].</t>
+          <t>This refund [TX-0083] was matched to the earlier charge [TX-0061] only because the merchant name is the same, and the amounts don't match, so it may be a partial refund or belong to a different booking. Check the merchant's booking details to confirm which charge [TX-0083] actually refunds before it is applied.</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -19989,23 +20283,23 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>TX-0067</t>
+          <t>TX-0089</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>TX-0067 · 2026-09-10 · TST* JOES PIZZA · USD 77.73 · Camila Ortiz · no receipt found in the matching window</t>
+          <t>TX-0089 · 2026-09-12 · TST* ZUMA MIAMI · USD 145.24 · Lucía Fernández · no receipt found in the matching window</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>No receipt was found for [TX-0067]. It stays in review until the cardholder uploads one.</t>
+          <t>The restaurant card charge [TX-0089] has no receipt in the matching window, so there is no support for the expense. Ask the cardholder for the receipt and confirm the business purpose before the charge is coded.</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -20017,28 +20311,28 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>missing_receipt</t>
+          <t>amount_mismatch</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>TX-0069</t>
+          <t>TX-0092</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>TX-0069 · 2026-09-10 · UBER *EATS HC9E7 · USD 50.39 · Tomás Herrera · no receipt found in the matching window</t>
+          <t>TX-0092 · 2026-09-12 · USDC PAYOUT LUCAS MOREAU · USDC 4,600.00 · receipt RC-0173 shows USDC 4,650.00 · difference USDC -50.00</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>No receipt was found for [TX-0069]. It stays in review until the cardholder uploads one.</t>
+          <t>The contractor payout [TX-0092] is a bit lower than the amount shown on its receipt [RC-0173], so they don't agree. Check whether [RC-0173] is a draft or estimate, then ask for the final receipt or record the difference with a note.</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -20055,23 +20349,23 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>TX-0071</t>
+          <t>TX-0115</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>TX-0071 · 2026-09-10 · UBER *TRIP T386M · USD 18.81 · Julián Castro · no receipt found in the matching window</t>
+          <t>TX-0115 · 2026-09-15 · SQ *BLUE BOTTLE COFFEE · USD 28.30 · Tomás Herrera · no receipt found in the matching window</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>No receipt was found for [TX-0071]. It stays in review until the cardholder uploads one.</t>
+          <t>No receipt was found for this coffee charge [TX-0115], so the business purpose rests only on the cardholder's memo. Ask the cardholder for the receipt and who the prospect was before accepting the suggested meals and representation account [AI-0012].</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -20083,28 +20377,28 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>amount_mismatch</t>
+          <t>duplicate_suspected</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>TX-0072</t>
+          <t>TX-0117</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>TX-0072 · 2026-09-10 · WEB SUMMIT RIO · USD 700.96 · Sofía Paz · receipt RC-0103 shows EUR 644.00 · different currency</t>
+          <t>TX-0117 · 2026-09-15 · STARBUCKS STORE YLFHT · USD 21.54 · Camila Ortiz · same descriptor and amount as TX-0104 posted 2026-09-14 · only one receipt</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>The receipt [RC-0103] matches [TX-0072] by merchant and date, but its amount or currency is different from the charge. The difference needs an explanation before posting.</t>
+          <t>[TX-0117] has the same merchant name and amount as [TX-0104] from the day before, and the lone receipt can support only one of them, so one may be a repeat charge. Check which charge the receipt matches and ask the cardholder whether both purchases were real before disputing.</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -20116,28 +20410,28 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>missing_receipt</t>
+          <t>duplicate_suspected</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>TX-0073</t>
+          <t>TX-0123</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>TX-0073 · 2026-09-11 · ATLASSIAN · USD 100.98 · Diego Romero · no receipt found in the matching window</t>
+          <t>TX-0123 · 2026-09-16 · ANTHROPIC · USD 222.25 · Diego Romero · same descriptor and amount as TX-0112 posted 2026-09-15 · only one receipt</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>No receipt was found for [TX-0073]. It stays in review until the cardholder uploads one.</t>
+          <t>[TX-0123] has the same merchant and amount as [TX-0112] from the day before, and only one receipt is on file, so it may be a repeat charge. Check with the cardholder whether both purchases were real, and only dispute [TX-0123] if the second one can't be supported.</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -20149,28 +20443,28 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>amount_mismatch</t>
+          <t>ai_below_threshold</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>TX-0079</t>
+          <t>TX-0127</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>TX-0079 · 2026-09-11 · MARRIOTT SAO PAULO · USD 333.76 · Valentina Sosa · receipt RC-0192 shows USD 293.76 · difference USD 40.00</t>
+          <t>TX-0127 · 2026-09-16 · SQ *SUNSET PRINT SHOP · USD 95.69 · Camila Ortiz · AI suggests 5.1.01 Publicidad y marketing with confidence 0.72 · threshold 0.75</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>The receipt [RC-0192] matches [TX-0079] by merchant and date, but its amount or currency is different from the charge. The difference needs an explanation before posting.</t>
+          <t>The suggestion [AI-0014] for marketing is below the confidence cutoff because the cardholder memo on [TX-0127] ("client meeting") doesn't obviously fit printed business cards. Check the receipt [RC-0050] and confirm whether marketing is the right account or whether office supplies or printing fits better.</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -20182,28 +20476,28 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>refund_partial_link</t>
+          <t>amount_mismatch</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>TX-0083</t>
+          <t>TX-0129</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>TX-0083 · 2026-09-12 · AIRBNB * HMM7983 · USD 111.51 · Diego Romero · tentatively linked to TX-0061 posted 2026-09-10 for USD 743.41 · amounts differ</t>
+          <t>TX-0129 · 2026-09-16 · TST* SHAKE SHACK MADISO · USD 126.55 · Camila Ortiz · receipt RC-0155 shows USD 110.22 · difference USD 16.33</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>[TX-0083] is a partial refund. It was linked to [TX-0061] because the merchant matches, but the amounts differ, so the link needs a person to confirm it.</t>
+          <t>The card charge [TX-0129] is higher than the receipt [RC-0155] matched to it, so the receipt may be a pre-tip or pre-final copy. Check whether a final itemized receipt exists, or whether the extra was a tip or added item, and confirm it fits the client meeting memo.</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -20215,28 +20509,28 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>missing_receipt</t>
+          <t>amount_mismatch</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>TX-0089</t>
+          <t>TX-0155</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>TX-0089 · 2026-09-12 · TST* ZUMA MIAMI · USD 145.24 · Lucía Fernández · no receipt found in the matching window</t>
+          <t>TX-0155 · 2026-09-19 · UDEMY ONLINE COURSE · USD 36.51 · Sofía Paz · receipt RC-0159 shows ARS 56,042.85 · different currency</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>No receipt was found for [TX-0089]. It stays in review until the cardholder uploads one.</t>
+          <t>The card charge [TX-0155] and the matched receipt [RC-0159] are in different currencies, so the amounts can't be compared directly. Check that [RC-0159] belongs to this purchase, then ask for the final receipt or record the currency difference.</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -20253,23 +20547,23 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>TX-0092</t>
+          <t>TX-0161</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>TX-0092 · 2026-09-12 · USDC PAYOUT LUCAS MOREAU · USDC 4,600.00 · receipt RC-0173 shows USDC 4,650.00 · difference USDC -50.00</t>
+          <t>TX-0161 · 2026-09-20 · TST* ZUMA MIAMI · USD 91.94 · Sofía Paz · receipt RC-0029 shows USD 80.07 · difference USD 11.87</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>The receipt [RC-0173] matches [TX-0092] by merchant and date, but its amount or currency is different from the charge. The difference needs an explanation before posting.</t>
+          <t>The card charge [TX-0161] is higher than the receipt [RC-0029] matched to it, so the receipt may be a pre-tip or itemized copy rather than the final one. Check whether the final receipt shows a tip or added items, and if not, ask Sofía Paz to explain the gap given the client meeting memo.</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -20281,28 +20575,28 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>no_rule</t>
+          <t>missing_receipt</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>TX-0111</t>
+          <t>TX-0162</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>TX-0111 · 2026-09-15 · AIRALO · USD 14.33 · Valentina Sosa · no account rule matches the descriptor</t>
+          <t>TX-0162 · 2026-09-20 · TWILIO FWB2B · USD 207.50 · Lucía Fernández · no receipt found in the matching window</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>No rule covers the merchant of [TX-0111].</t>
+          <t>No receipt was found for the Twilio card charge [TX-0162], so the actual service bought is unconfirmed. Ask the cardholder for the receipt and check that it supports the cloud services account suggested in [AI-0018] before accepting it.</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -20319,23 +20613,23 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>TX-0115</t>
+          <t>TX-0165</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>TX-0115 · 2026-09-15 · SQ *BLUE BOTTLE COFFEE · USD 28.30 · Tomás Herrera · no receipt found in the matching window</t>
+          <t>TX-0165 · 2026-09-20 · UBER *TRIP AXJQT · USD 15.30 · Lucía Fernández · no receipt found in the matching window</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>No receipt was found for [TX-0115]. It stays in review until the cardholder uploads one.</t>
+          <t>The ride-share charge [TX-0165] on Lucía Fernández's card has no receipt in the matching window. Ask her for the receipt and check that the trip was for business.</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -20347,28 +20641,28 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>no_rule</t>
+          <t>amount_mismatch</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>TX-0115</t>
+          <t>TX-0168</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>TX-0115 · 2026-09-15 · SQ *BLUE BOTTLE COFFEE · USD 28.30 · Tomás Herrera · no account rule matches the descriptor</t>
+          <t>TX-0168 · 2026-09-21 · HILTON MIAMI DOWNTOWN · USD 984.99 · Julián Castro · receipt RC-0210 shows USD 899.99 · difference USD 85.00</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>No rule covers the merchant of [TX-0115].</t>
+          <t>The card charge [TX-0168] from the Hilton is higher than the amount on the matched receipt [RC-0210]. Check whether [RC-0210] is a preliminary bill and ask Julián for the final receipt, or confirm what the extra charge covers (for example incidentals) before recording the difference.</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -20380,28 +20674,28 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>no_rule</t>
+          <t>missing_receipt</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>TX-0116</t>
+          <t>TX-0179</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>TX-0116 · 2026-09-15 · SQ *BLUE BOTTLE COFFEE · USD 38.21 · Martín Ibarra · no account rule matches the descriptor</t>
+          <t>TX-0179 · 2026-09-22 · MARRIOTT SAO PAULO · USD 470.08 · Lucía Fernández · no receipt found in the matching window</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>No rule covers the merchant of [TX-0116].</t>
+          <t>The hotel charge [TX-0179] on Lucía Fernández's card has no matching receipt in the search window. Ask her for the receipt, and check whether it was filed late or under a different date or amount.</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -20413,28 +20707,28 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>duplicate_suspected</t>
+          <t>missing_receipt</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>TX-0117</t>
+          <t>TX-0188</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>TX-0117 · 2026-09-15 · STARBUCKS STORE YLFHT · USD 21.54 · Camila Ortiz · same descriptor and amount as TX-0104 posted 2026-09-14 · only one receipt</t>
+          <t>TX-0188 · 2026-09-23 · STICKERMULE.COM · USD 398.16 · Tomás Herrera · no receipt found in the matching window</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>[TX-0117] repeats the merchant and amount of [TX-0104] within a short window, and only one receipt exists. It looks like a double charge.</t>
+          <t>No receipt was found for the Sticker Mule card charge [TX-0188], so what was bought and why is unconfirmed. Ask the cardholder for the receipt and confirm it was a business purchase before accepting the marketing account suggested in [AI-0023], which is only a guess from the merchant name.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -20446,28 +20740,28 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>duplicate_suspected</t>
+          <t>ai_below_threshold</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>TX-0123</t>
+          <t>TX-0188</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>TX-0123 · 2026-09-16 · ANTHROPIC · USD 222.25 · Diego Romero · same descriptor and amount as TX-0112 posted 2026-09-15 · only one receipt</t>
+          <t>TX-0188 · 2026-09-23 · STICKERMULE.COM · USD 398.16 · Tomás Herrera · AI suggests 5.1.01 Publicidad y marketing with confidence 0.60 · threshold 0.75</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>[TX-0123] repeats the merchant and amount of [TX-0112] within a short window, and only one receipt exists. It looks like a double charge.</t>
+          <t>The AI's marketing suggestion [AI-0023] for this Sticker Mule charge [TX-0188] is low confidence, and there is no receipt or memo to show what was bought. Ask the cardholder what the items were, then pick the account yourself, since the stickers could be marketing or something else.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -20479,28 +20773,28 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>no_rule</t>
+          <t>refund_partial_link</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>TX-0127</t>
+          <t>TX-0198</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>TX-0127 · 2026-09-16 · SQ *SUNSET PRINT SHOP · USD 95.69 · Camila Ortiz · no account rule matches the descriptor</t>
+          <t>TX-0198 · 2026-09-24 · LATAM AIRLINES B2LK8 · USD 38.00 · Lucía Fernández · tentatively linked to TX-0169 posted 2026-09-21 for USD 316.74 · amounts differ</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>No rule covers the merchant of [TX-0127].</t>
+          <t>This refund [TX-0198] was matched to the earlier charge [TX-0169] only because the merchant is the same, and the amounts don't match, so it may be a partial refund or belong to a different booking. Check the airline booking reference and ticket details to confirm which charge [TX-0198] actually refunds.</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -20512,28 +20806,28 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>amount_mismatch</t>
+          <t>missing_receipt</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>TX-0129</t>
+          <t>TX-0201</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>TX-0129 · 2026-09-16 · TST* SHAKE SHACK MADISO · USD 126.55 · Camila Ortiz · receipt RC-0155 shows USD 110.22 · difference USD 16.33</t>
+          <t>TX-0201 · 2026-09-24 · UBER *TRIP GFDW2 · USD 29.25 · Lucía Fernández · no receipt found in the matching window</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>The receipt [RC-0155] matches [TX-0129] by merchant and date, but its amount or currency is different from the charge. The difference needs an explanation before posting.</t>
+          <t>The ride charge [TX-0201] has no receipt in the matching window, so there is nothing to support it yet. Ask the cardholder for the receipt and check that the trip was for business.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -20545,28 +20839,28 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>no_rule</t>
+          <t>missing_receipt</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>TX-0134</t>
+          <t>TX-0203</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>TX-0134 · 2026-09-17 · DUTY FREE AMERICAS 23MZD · USD 142.45 · Camila Ortiz · no account rule matches the descriptor</t>
+          <t>TX-0203 · 2026-09-25 · FACEBK *ADS TKMC3 · USD 202.68 · Camila Ortiz · no receipt found in the matching window</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>No rule covers the merchant of [TX-0134].</t>
+          <t>This Facebook ads charge [TX-0203] on Camila Ortiz's card has no receipt in the matching window. Ask the cardholder for the receipt, and check whether the ad platform's billing page shows a matching invoice that was filed elsewhere.</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -20578,28 +20872,28 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>no_rule</t>
+          <t>amount_mismatch</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>TX-0142</t>
+          <t>TX-0205</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>TX-0142 · 2026-09-18 · UPWORK *ESCROW RHX2D · USD 683.64 · Julián Castro · no account rule matches the descriptor</t>
+          <t>TX-0205 · 2026-09-25 · TST* ZUMA MIAMI · USD 55.39 · Valentina Sosa · receipt RC-0125 shows USD 48.24 · difference USD 7.15</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>No rule covers the merchant of [TX-0142].</t>
+          <t>The card charge [TX-0205] is higher than the receipt [RC-0125] attached to it, which may mean a tip was added after the receipt was printed or the wrong receipt was matched. Check whether [RC-0125] is the final itemized receipt for this meal, and if so, ask the cardholder for the final copy or record the difference.</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -20611,28 +20905,28 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>amount_mismatch</t>
+          <t>missing_receipt</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>TX-0155</t>
+          <t>TX-0208</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>TX-0155 · 2026-09-19 · UDEMY ONLINE COURSE · USD 36.51 · Sofía Paz · receipt RC-0159 shows ARS 56,042.85 · different currency</t>
+          <t>TX-0208 · 2026-09-26 · DD *DOORDASH DEHYT · USD 132.46 · Tomás Herrera · no receipt found in the matching window</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>The receipt [RC-0159] matches [TX-0155] by merchant and date, but its amount or currency is different from the charge. The difference needs an explanation before posting.</t>
+          <t>No receipt was found for this food delivery charge [TX-0208], so the team dinner described in the memo can't be confirmed. Ask the cardholder for the receipt, and check it supports the suggested meals and entertainment account [AI-0026] before anything is coded.</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -20644,28 +20938,28 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>no_rule</t>
+          <t>duplicate_suspected</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>TX-0156</t>
+          <t>TX-0211</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>TX-0156 · 2026-09-20 · BEST BUY 00012 · USD 94.38 · Sofía Paz · no account rule matches the descriptor</t>
+          <t>TX-0211 · 2026-09-26 · STARBUCKS STORE DEC7E · USD 26.63 · Valentina Sosa · same descriptor and amount as TX-0210 posted 2026-09-26 · only one receipt</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>No rule covers the merchant of [TX-0156].</t>
+          <t>[TX-0211] has the same merchant descriptor and amount as [TX-0210] on the same day, and only one receipt exists, so it may be a repeat charge. Ask the cardholder whether both purchases were real, and check the receipt against both before deciding whether to dispute.</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -20677,28 +20971,28 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>amount_mismatch</t>
+          <t>ai_below_threshold</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>TX-0161</t>
+          <t>TX-0214</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>TX-0161 · 2026-09-20 · TST* ZUMA MIAMI · USD 91.94 · Sofía Paz · receipt RC-0029 shows USD 80.07 · difference USD 11.87</t>
+          <t>TX-0214 · 2026-09-27 · APPLE.COM/BILL · USD 9.99 · Julián Castro · AI suggests 5.1.03 Licencias de software with confidence 0.72 · threshold 0.75</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>The receipt [RC-0029] matches [TX-0161] by merchant and date, but its amount or currency is different from the charge. The difference needs an explanation before posting.</t>
+          <t>The AI's account suggestion [AI-0027] for this card charge [TX-0214] falls just short of the confidence bar, so it needs a person to choose. The receipt [RC-0046] reads like a flat-fee software subscription, but check that the other account the AI named is not a better fit before you pick.</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -20710,28 +21004,28 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>missing_receipt</t>
+          <t>duplicate_suspected</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>TX-0162</t>
+          <t>TX-0217</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>TX-0162 · 2026-09-20 · TWILIO FWB2B · USD 207.50 · Lucía Fernández · no receipt found in the matching window</t>
+          <t>TX-0217 · 2026-09-27 · TST* JOES PIZZA · USD 88.24 · Martín Ibarra · same descriptor and amount as TX-0216 posted 2026-09-27 · only one receipt</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>No receipt was found for [TX-0162]. It stays in review until the cardholder uploads one.</t>
+          <t>[TX-0217] has the same merchant and amount as [TX-0216] on the same day, yet only one receipt is on file. Check with the cardholder whether both purchases were real, and if not, dispute [TX-0217].</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -20743,28 +21037,28 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>no_rule</t>
+          <t>missing_receipt</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>TX-0162</t>
+          <t>TX-0236</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>TX-0162 · 2026-09-20 · TWILIO FWB2B · USD 207.50 · Lucía Fernández · no account rule matches the descriptor</t>
+          <t>TX-0236 · 2026-09-29 · USDC PAYOUT LUCAS MOREAU · USDC 4,700.00 · no receipt found in the matching window</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>No rule covers the merchant of [TX-0162].</t>
+          <t>The stablecoin payout to the contractor in [TX-0236] has no receipt or invoice in the matching window, so there is no support for it. Ask the contractor for the invoice and check whether it was filed under a different date or payment.</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>
@@ -20776,820 +21070,28 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>TX-0165</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr"/>
+          <t>receipt_unmatched</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>RC-0211</t>
+        </is>
+      </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>TX-0165 · 2026-09-20 · UBER *TRIP AXJQT · USD 15.30 · Lucía Fernández · no receipt found in the matching window</t>
+          <t>RC-0211 · Uber Portier B.V. · 2026-09-09 · ARS 77,348.65</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>No receipt was found for [TX-0165]. It stays in review until the cardholder uploads one.</t>
+          <t>Receipt [RC-0211] from Uber Portier B.V. has no matching card transaction in the ledger. Check whether the charge posted under a different date, amount or merchant name, or was paid another way; if nothing turns up, discard the receipt.</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>template</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>EX-045</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>TX-0167</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>TX-0167 · 2026-09-21 · AMZN MKTP US*H7N3G · USD 149.83 · Valentina Sosa · no account rule matches the descriptor</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>No rule covers the merchant of [TX-0167].</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>EX-046</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>amount_mismatch</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>TX-0168</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>TX-0168 · 2026-09-21 · HILTON MIAMI DOWNTOWN · USD 984.99 · Julián Castro · receipt RC-0210 shows USD 899.99 · difference USD 85.00</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>The receipt [RC-0210] matches [TX-0168] by merchant and date, but its amount or currency is different from the charge. The difference needs an explanation before posting.</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>EX-047</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>TX-0170</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>TX-0170 · 2026-09-21 · LEMSQZY* TAILWIND LABS · USD 299.00 · Martín Ibarra · no account rule matches the descriptor</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>No rule covers the merchant of [TX-0170].</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>EX-048</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>TX-0171</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>TX-0171 · 2026-09-21 · LYFT *RIDE WV4T9 · USD 21.09 · Lucía Fernández · no account rule matches the descriptor</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>No rule covers the merchant of [TX-0171].</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>EX-049</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>TX-0178</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>TX-0178 · 2026-09-22 · LYFT *RIDE J7H7L · USD 34.76 · Diego Romero · no account rule matches the descriptor</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>No rule covers the merchant of [TX-0178].</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>EX-050</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>TX-0179</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>TX-0179 · 2026-09-22 · MARRIOTT SAO PAULO · USD 470.08 · Lucía Fernández · no receipt found in the matching window</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>No receipt was found for [TX-0179]. It stays in review until the cardholder uploads one.</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>EX-051</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>TX-0188</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>TX-0188 · 2026-09-23 · STICKERMULE.COM · USD 398.16 · Tomás Herrera · no receipt found in the matching window</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>No receipt was found for [TX-0188]. It stays in review until the cardholder uploads one.</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>EX-052</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>TX-0188</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>TX-0188 · 2026-09-23 · STICKERMULE.COM · USD 398.16 · Tomás Herrera · no account rule matches the descriptor</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>No rule covers the merchant of [TX-0188].</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>EX-053</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>TX-0189</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>TX-0189 · 2026-09-23 · TICKETTAILOR* PRODUCTCAMP · USD 48.29 · Diego Romero · no account rule matches the descriptor</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>No rule covers the merchant of [TX-0189].</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>EX-054</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>TX-0195</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>TX-0195 · 2026-09-24 · COSTCO WHSE #0144 · USD 141.72 · Sofía Paz · no account rule matches the descriptor</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>No rule covers the merchant of [TX-0195].</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>EX-055</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>refund_partial_link</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>TX-0198</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>TX-0198 · 2026-09-24 · LATAM AIRLINES B2LK8 · USD 38.00 · Lucía Fernández · tentatively linked to TX-0169 posted 2026-09-21 for USD 316.74 · amounts differ</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>[TX-0198] is a partial refund. It was linked to [TX-0169] because the merchant matches, but the amounts differ, so the link needs a person to confirm it.</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>EX-056</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>TX-0201</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>TX-0201 · 2026-09-24 · UBER *TRIP GFDW2 · USD 29.25 · Lucía Fernández · no receipt found in the matching window</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>No receipt was found for [TX-0201]. It stays in review until the cardholder uploads one.</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>EX-057</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>TX-0203</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>TX-0203 · 2026-09-25 · FACEBK *ADS TKMC3 · USD 202.68 · Camila Ortiz · no receipt found in the matching window</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>No receipt was found for [TX-0203]. It stays in review until the cardholder uploads one.</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>EX-058</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>amount_mismatch</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>TX-0205</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr"/>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>TX-0205 · 2026-09-25 · TST* ZUMA MIAMI · USD 55.39 · Valentina Sosa · receipt RC-0125 shows USD 48.24 · difference USD 7.15</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>The receipt [RC-0125] matches [TX-0205] by merchant and date, but its amount or currency is different from the charge. The difference needs an explanation before posting.</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>EX-059</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>TX-0208</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>TX-0208 · 2026-09-26 · DD *DOORDASH DEHYT · USD 132.46 · Tomás Herrera · no receipt found in the matching window</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>No receipt was found for [TX-0208]. It stays in review until the cardholder uploads one.</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>EX-060</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>TX-0208</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>TX-0208 · 2026-09-26 · DD *DOORDASH DEHYT · USD 132.46 · Tomás Herrera · no account rule matches the descriptor</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>No rule covers the merchant of [TX-0208].</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>EX-061</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>duplicate_suspected</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>TX-0211</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>TX-0211 · 2026-09-26 · STARBUCKS STORE DEC7E · USD 26.63 · Valentina Sosa · same descriptor and amount as TX-0210 posted 2026-09-26 · only one receipt</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>[TX-0211] repeats the merchant and amount of [TX-0210] within a short window, and only one receipt exists. It looks like a double charge.</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>EX-062</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>TX-0214</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>TX-0214 · 2026-09-27 · APPLE.COM/BILL · USD 9.99 · Julián Castro · no account rule matches the descriptor</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>No rule covers the merchant of [TX-0214].</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>EX-063</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>duplicate_suspected</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>TX-0217</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>TX-0217 · 2026-09-27 · TST* JOES PIZZA · USD 88.24 · Martín Ibarra · same descriptor and amount as TX-0216 posted 2026-09-27 · only one receipt</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>[TX-0217] repeats the merchant and amount of [TX-0216] within a short window, and only one receipt exists. It looks like a double charge.</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>EX-064</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>TX-0229</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr"/>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>TX-0229 · 2026-09-29 · SENDGRID · USD 90.00 · Lucía Fernández · no account rule matches the descriptor</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>No rule covers the merchant of [TX-0229].</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>EX-065</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>TX-0236</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr"/>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>TX-0236 · 2026-09-29 · USDC PAYOUT LUCAS MOREAU · USDC 4,700.00 · no receipt found in the matching window</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>No receipt was found for [TX-0236]. It stays in review until the cardholder uploads one.</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>EX-066</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>TX-0239</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>TX-0239 · 2026-09-30 · AMZN MKTP US*D8TEW · USD 29.62 · Diego Romero · no account rule matches the descriptor</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>No rule covers the merchant of [TX-0239].</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>EX-067</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>no_rule</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>TX-0244</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>TX-0244 · 2026-09-30 · TWILIO 2NWKH · USD 158.45 · Camila Ortiz · no account rule matches the descriptor</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>No rule covers the merchant of [TX-0244].</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>EX-068</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>receipt_unmatched</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr"/>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>RC-0211</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>RC-0211 · Uber Portier B.V. · 2026-09-09 · ARS 77,348.65</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>The receipt [RC-0211] did not match any transaction in the export.</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>template</t>
+          <t>ai_verified</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Value USDC at the crypto dollar rate, repost to the QuickBooks sandbox
USDC payouts, top ups, the opening balance and the month end remeasurement
now use the crypto dollar seller rate from the snapshot. Dollar card spend
stays at the official rate. Paying the card with USDC moves the gap to
exchange differences. Methodology, Excel, page and README updated. The
sandbox entry CTL-2026-09 was deleted by hand and posted again: 512 lines,
verified to the cent.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/out/cierre_2026-09_andes_labs.xlsx
+++ b/data/out/cierre_2026-09_andes_labs.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>203535812.05</v>
+        <v>208711799.05</v>
       </c>
     </row>
     <row r="10">
@@ -611,6 +611,16 @@
       </c>
       <c r="B16" t="n">
         <v>1545</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Tipo de cambio de cierre USDC (dólar cripto vendedor)</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1612.31</v>
       </c>
     </row>
   </sheetData>
@@ -688,7 +698,7 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>10315172.7</v>
+        <v>10887596.18</v>
       </c>
     </row>
     <row r="4">
@@ -703,7 +713,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>22744110.4</v>
+        <v>23373642.4</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>0</v>
@@ -793,7 +803,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>105067844</v>
+        <v>109614299</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>0</v>
@@ -919,7 +929,7 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>4781167.65</v>
+        <v>177604.13</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>0</v>
@@ -933,10 +943,10 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>208316979.7</v>
+        <v>208889403.18</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>208316979.7</v>
+        <v>208889403.18</v>
       </c>
     </row>
   </sheetData>
@@ -1673,7 +1683,7 @@
         <v>60000000</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>1535</v>
+        <v>1586.98</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>60000000</v>
@@ -3282,7 +3292,7 @@
         <v>1530</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>63092885.4</v>
+        <v>64954744.08</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -7768,10 +7778,10 @@
         <v>4600</v>
       </c>
       <c r="G93" s="2" t="n">
-        <v>1530</v>
+        <v>1594.25</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>7038000</v>
+        <v>7333550</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>
@@ -9086,7 +9096,7 @@
         <v>45000000</v>
       </c>
       <c r="G111" s="2" t="n">
-        <v>1530</v>
+        <v>1593.47</v>
       </c>
       <c r="H111" s="2" t="n">
         <v>45000000</v>
@@ -9897,10 +9907,10 @@
         <v>5450</v>
       </c>
       <c r="G122" s="2" t="n">
-        <v>1530</v>
+        <v>1593.47</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>8338500</v>
+        <v>8684411.5</v>
       </c>
       <c r="I122" t="inlineStr">
         <is>
@@ -9970,10 +9980,10 @@
         <v>4200</v>
       </c>
       <c r="G123" s="2" t="n">
-        <v>1530</v>
+        <v>1593.47</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>6426000</v>
+        <v>6692574</v>
       </c>
       <c r="I123" t="inlineStr">
         <is>
@@ -14479,10 +14489,10 @@
         <v>5050</v>
       </c>
       <c r="G184" s="2" t="n">
-        <v>1535</v>
+        <v>1594.83</v>
       </c>
       <c r="H184" s="2" t="n">
-        <v>7751750</v>
+        <v>8053891.5</v>
       </c>
       <c r="I184" t="inlineStr">
         <is>
@@ -17784,7 +17794,7 @@
         <v>70000000</v>
       </c>
       <c r="G229" s="2" t="n">
-        <v>1545</v>
+        <v>1616.06</v>
       </c>
       <c r="H229" s="2" t="n">
         <v>70000000</v>
@@ -18003,10 +18013,10 @@
         <v>3600</v>
       </c>
       <c r="G232" s="2" t="n">
-        <v>1545</v>
+        <v>1616.06</v>
       </c>
       <c r="H232" s="2" t="n">
-        <v>5562000</v>
+        <v>5817816</v>
       </c>
       <c r="I232" t="inlineStr">
         <is>
@@ -18076,10 +18086,10 @@
         <v>3300</v>
       </c>
       <c r="G233" s="2" t="n">
-        <v>1545</v>
+        <v>1616.06</v>
       </c>
       <c r="H233" s="2" t="n">
-        <v>5098500</v>
+        <v>5332998</v>
       </c>
       <c r="I233" t="inlineStr">
         <is>
@@ -18149,10 +18159,10 @@
         <v>2900</v>
       </c>
       <c r="G234" s="2" t="n">
-        <v>1545</v>
+        <v>1616.06</v>
       </c>
       <c r="H234" s="2" t="n">
-        <v>4480500</v>
+        <v>4686574</v>
       </c>
       <c r="I234" t="inlineStr">
         <is>
@@ -18222,10 +18232,10 @@
         <v>2800</v>
       </c>
       <c r="G235" s="2" t="n">
-        <v>1545</v>
+        <v>1616.06</v>
       </c>
       <c r="H235" s="2" t="n">
-        <v>4326000</v>
+        <v>4524968</v>
       </c>
       <c r="I235" t="inlineStr">
         <is>
@@ -18295,10 +18305,10 @@
         <v>3000</v>
       </c>
       <c r="G236" s="2" t="n">
-        <v>1545</v>
+        <v>1616.06</v>
       </c>
       <c r="H236" s="2" t="n">
-        <v>4635000</v>
+        <v>4848180</v>
       </c>
       <c r="I236" t="inlineStr">
         <is>
@@ -18368,10 +18378,10 @@
         <v>4700</v>
       </c>
       <c r="G237" s="2" t="n">
-        <v>1545</v>
+        <v>1616.06</v>
       </c>
       <c r="H237" s="2" t="n">
-        <v>7261500</v>
+        <v>7595482</v>
       </c>
       <c r="I237" t="inlineStr">
         <is>
@@ -18441,10 +18451,10 @@
         <v>5200</v>
       </c>
       <c r="G238" s="2" t="n">
-        <v>1545</v>
+        <v>1616.06</v>
       </c>
       <c r="H238" s="2" t="n">
-        <v>8034000</v>
+        <v>8403512</v>
       </c>
       <c r="I238" t="inlineStr">
         <is>
@@ -18514,10 +18524,10 @@
         <v>4450</v>
       </c>
       <c r="G239" s="2" t="n">
-        <v>1545</v>
+        <v>1616.06</v>
       </c>
       <c r="H239" s="2" t="n">
-        <v>6875250</v>
+        <v>7191467</v>
       </c>
       <c r="I239" t="inlineStr">
         <is>
@@ -19029,10 +19039,10 @@
         <v>2700</v>
       </c>
       <c r="G246" s="2" t="n">
-        <v>1545</v>
+        <v>1612.31</v>
       </c>
       <c r="H246" s="2" t="n">
-        <v>4171500</v>
+        <v>4353237</v>
       </c>
       <c r="I246" t="inlineStr">
         <is>
@@ -19102,10 +19112,10 @@
         <v>4100</v>
       </c>
       <c r="G247" s="2" t="n">
-        <v>1545</v>
+        <v>1612.31</v>
       </c>
       <c r="H247" s="2" t="n">
-        <v>6334500</v>
+        <v>6610471</v>
       </c>
       <c r="I247" t="inlineStr">
         <is>
@@ -19175,10 +19185,10 @@
         <v>2500</v>
       </c>
       <c r="G248" s="2" t="n">
-        <v>1545</v>
+        <v>1612.31</v>
       </c>
       <c r="H248" s="2" t="n">
-        <v>3862500</v>
+        <v>4030775</v>
       </c>
       <c r="I248" t="inlineStr">
         <is>
@@ -19248,10 +19258,10 @@
         <v>3900</v>
       </c>
       <c r="G249" s="2" t="n">
-        <v>1545</v>
+        <v>1612.31</v>
       </c>
       <c r="H249" s="2" t="n">
-        <v>6025500</v>
+        <v>6288009</v>
       </c>
       <c r="I249" t="inlineStr">
         <is>
@@ -19321,10 +19331,10 @@
         <v>4650</v>
       </c>
       <c r="G250" s="2" t="n">
-        <v>1545</v>
+        <v>1612.31</v>
       </c>
       <c r="H250" s="2" t="n">
-        <v>7184250</v>
+        <v>7497241.5</v>
       </c>
       <c r="I250" t="inlineStr">
         <is>
@@ -19394,10 +19404,10 @@
         <v>3400</v>
       </c>
       <c r="G251" s="2" t="n">
-        <v>1545</v>
+        <v>1612.31</v>
       </c>
       <c r="H251" s="2" t="n">
-        <v>5253000</v>
+        <v>5481854</v>
       </c>
       <c r="I251" t="inlineStr">
         <is>
@@ -19467,10 +19477,10 @@
         <v>2700</v>
       </c>
       <c r="G252" s="2" t="n">
-        <v>1545</v>
+        <v>1612.31</v>
       </c>
       <c r="H252" s="2" t="n">
-        <v>4171500</v>
+        <v>4353237</v>
       </c>
       <c r="I252" t="inlineStr">
         <is>
@@ -19540,10 +19550,10 @@
         <v>3350</v>
       </c>
       <c r="G253" s="2" t="n">
-        <v>1545</v>
+        <v>1612.31</v>
       </c>
       <c r="H253" s="2" t="n">
-        <v>5175750</v>
+        <v>5401238.5</v>
       </c>
       <c r="I253" t="inlineStr">
         <is>
@@ -21161,7 +21171,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Official seller rate (venta) on the posting date of each movement. To validate with an accountant: buyer rate for assets, transaction date versus posting date, and Banco Nación versus BCRA Comunicación A 3500.</t>
+          <t>Seller rate (venta) on the posting date of each movement: official for dollar card spend, crypto dollar for USDC. To validate with an accountant: buyer rate for assets, transaction date versus posting date, and Banco Nación versus BCRA Comunicación A 3500.</t>
         </is>
       </c>
     </row>
@@ -21195,7 +21205,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>One USDC is treated as one US dollar at the official rate. Whether USDC should be valued at the official, MEP or crypto rate is an open question for the accountant.</t>
+          <t>USDC is valued at the crypto dollar seller rate of each day (https://api.argentinadatos.com/v1/cotizaciones/dolares/cripto), the rate at which it can be turned into pesos. One USDC is treated as one crypto dollar. Dollar card spend stays at the official rate. Whether USDC should be valued at the crypto, MEP or official rate is a question for the accountant.</t>
         </is>
       </c>
     </row>
@@ -21212,7 +21222,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>USDC received is computed from the ARS sent at the crypto dollar seller rate of that day (https://api.argentinadatos.com/v1/cotizaciones/dolares/cripto). The gap against the official rate goes to Diferencias de cambio.</t>
+          <t>USDC received is computed from the ARS sent at the crypto dollar seller rate of that day and booked at the same rate. Only the rounding the exchange keeps goes to Diferencias de cambio.</t>
         </is>
       </c>
     </row>
@@ -21229,7 +21239,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Cuenta USDC and Tarjeta corporativa a pagar are remeasured at the official seller rate of the last day of the month. The difference goes to Diferencias de cambio.</t>
+          <t>Cuenta USDC is remeasured at the crypto dollar seller rate of the last day of the month and Tarjeta corporativa a pagar at the official seller rate of that day. Paying the card with USDC moves the gap between the two rates to Diferencias de cambio, and so does each remeasurement.</t>
         </is>
       </c>
     </row>
@@ -21246,7 +21256,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Synthetic opening balances as of 2026-08-31, valued at that day's official seller rate.</t>
+          <t>Synthetic opening balances as of 2026-08-31, valued at that day's crypto seller rate for USDC and official seller rate for the card payable.</t>
         </is>
       </c>
     </row>

</xml_diff>